<commit_message>
Remove answer-control language from SQLite audit task
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R9fbb479da49e47ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R1701e5fd60394aa2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -466,7 +466,7 @@
         <x:v>审计摘要</x:v>
       </x:c>
       <x:c r="B14" s="21" t="str">
-        <x:v>audit_summary汇总源数据量、有效线程、异常、规则、SLA和自动升级控制量，并检查队列映射、异常隔离及线程与SLA根集合一致性</x:v>
+        <x:v>audit_summary汇总数据截止时间、源数据量、有效线程、异常、规则、SLA和自动升级次数</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="56" customHeight="1">
@@ -474,7 +474,7 @@
         <x:v>运行边界</x:v>
       </x:c>
       <x:c r="B15" s="21" t="str">
-        <x:v>npm run audit调用真实SQLite CLI；输入数据库和规则文件保持只读，SQL执行未成功时不保留未完成的数据库与报告</x:v>
+        <x:v>npm run audit调用真实SQLite CLI；输入数据库和规则文件保持只读，结果写入output目录</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
@@ -487,7 +487,7 @@
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
       <x:c r="A17" s="14" t="str">
-        <x:v>可验证点</x:v>
+        <x:v>业务核对点</x:v>
       </x:c>
       <x:c r="B17" s="21" t="str">
         <x:v>SQLite进程与版本；三份业务输入的读取；递归父链结果；json_each展开；队列映射；unixepoch时间差；五张派生表；四份CSV与审计JSON的跨文件对应</x:v>

</xml_diff>